<commit_message>
Training 8 oktober toegevoegd
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/WB3 Stats.xlsx
+++ b/data/WB3 Stats.xlsx
@@ -1923,7 +1923,9 @@
       <c r="F2" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G2" s="7" t="n"/>
+      <c r="G2" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="H2" s="7" t="n"/>
       <c r="I2" s="7" t="n"/>
       <c r="J2" s="7" t="n"/>
@@ -1955,7 +1957,9 @@
       <c r="F3" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="7" t="n"/>
+      <c r="G3" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H3" s="7" t="n"/>
       <c r="I3" s="7" t="n"/>
       <c r="J3" s="7" t="n"/>
@@ -1987,7 +1991,9 @@
       <c r="F4" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="7" t="n"/>
+      <c r="G4" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H4" s="7" t="n"/>
       <c r="I4" s="7" t="n"/>
       <c r="J4" s="7" t="n"/>
@@ -2019,7 +2025,9 @@
       <c r="F5" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="7" t="n"/>
+      <c r="G5" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H5" s="7" t="n"/>
       <c r="I5" s="7" t="n"/>
       <c r="J5" s="7" t="n"/>
@@ -2051,7 +2059,9 @@
       <c r="F6" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="7" t="n"/>
+      <c r="G6" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
       <c r="J6" s="7" t="n"/>
@@ -2083,7 +2093,9 @@
       <c r="F7" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="7" t="n"/>
+      <c r="G7" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="H7" s="7" t="n"/>
       <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="n"/>
@@ -2115,7 +2127,9 @@
       <c r="F8" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="7" t="n"/>
+      <c r="G8" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H8" s="7" t="n"/>
       <c r="I8" s="7" t="n"/>
       <c r="J8" s="7" t="n"/>
@@ -2147,7 +2161,9 @@
       <c r="F9" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="7" t="n"/>
+      <c r="G9" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H9" s="7" t="n"/>
       <c r="I9" s="7" t="n"/>
       <c r="J9" s="7" t="n"/>
@@ -2179,7 +2195,9 @@
       <c r="F10" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="7" t="n"/>
+      <c r="G10" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H10" s="7" t="n"/>
       <c r="I10" s="7" t="n"/>
       <c r="J10" s="7" t="n"/>
@@ -2211,7 +2229,9 @@
       <c r="F11" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="7" t="n"/>
+      <c r="G11" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H11" s="7" t="n"/>
       <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="n"/>
@@ -2243,7 +2263,9 @@
       <c r="F12" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="7" t="n"/>
+      <c r="G12" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="H12" s="7" t="n"/>
       <c r="I12" s="7" t="n"/>
       <c r="J12" s="7" t="n"/>
@@ -2275,7 +2297,9 @@
       <c r="F13" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="7" t="n"/>
+      <c r="G13" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H13" s="7" t="n"/>
       <c r="I13" s="7" t="n"/>
       <c r="J13" s="7" t="n"/>
@@ -2307,7 +2331,9 @@
       <c r="F14" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="7" t="n"/>
+      <c r="G14" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H14" s="7" t="n"/>
       <c r="I14" s="7" t="n"/>
       <c r="J14" s="7" t="n"/>
@@ -2339,7 +2365,9 @@
       <c r="F15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="7" t="n"/>
+      <c r="G15" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H15" s="7" t="n"/>
       <c r="I15" s="7" t="n"/>
       <c r="J15" s="7" t="n"/>
@@ -2371,7 +2399,9 @@
       <c r="F16" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G16" s="7" t="n"/>
+      <c r="G16" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="H16" s="7" t="n"/>
       <c r="I16" s="7" t="n"/>
       <c r="J16" s="7" t="n"/>
@@ -2403,7 +2433,9 @@
       <c r="F17" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G17" s="7" t="n"/>
+      <c r="G17" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H17" s="7" t="n"/>
       <c r="I17" s="7" t="n"/>
       <c r="J17" s="7" t="n"/>
@@ -2435,7 +2467,9 @@
       <c r="F18" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G18" s="7" t="n"/>
+      <c r="G18" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="H18" s="7" t="n"/>
       <c r="I18" s="7" t="n"/>
       <c r="J18" s="7" t="n"/>
@@ -2467,7 +2501,9 @@
       <c r="F19" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G19" s="7" t="n"/>
+      <c r="G19" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H19" s="7" t="n"/>
       <c r="I19" s="7" t="n"/>
       <c r="J19" s="7" t="n"/>
@@ -2499,7 +2535,9 @@
       <c r="F20" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="7" t="n"/>
+      <c r="G20" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="H20" s="7" t="n"/>
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="7" t="n"/>
@@ -2531,7 +2569,9 @@
       <c r="F21" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G21" s="7" t="n"/>
+      <c r="G21" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H21" s="7" t="n"/>
       <c r="I21" s="7" t="n"/>
       <c r="J21" s="7" t="n"/>
@@ -2563,7 +2603,9 @@
       <c r="F22" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G22" s="7" t="n"/>
+      <c r="G22" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H22" s="7" t="n"/>
       <c r="I22" s="7" t="n"/>
       <c r="J22" s="7" t="n"/>
@@ -2595,7 +2637,9 @@
       <c r="F23" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G23" s="7" t="n"/>
+      <c r="G23" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H23" s="7" t="n"/>
       <c r="I23" s="7" t="n"/>
       <c r="J23" s="7" t="n"/>
@@ -2627,7 +2671,9 @@
       <c r="F24" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G24" s="7" t="n"/>
+      <c r="G24" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H24" s="7" t="n"/>
       <c r="I24" s="7" t="n"/>
       <c r="J24" s="7" t="n"/>
@@ -2659,7 +2705,9 @@
       <c r="F25" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="7" t="n"/>
+      <c r="G25" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="H25" s="7" t="n"/>
       <c r="I25" s="7" t="n"/>
       <c r="J25" s="7" t="n"/>
@@ -2691,7 +2739,9 @@
       <c r="F26" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G26" s="7" t="n"/>
+      <c r="G26" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H26" s="7" t="n"/>
       <c r="I26" s="7" t="n"/>
       <c r="J26" s="7" t="n"/>
@@ -2723,7 +2773,9 @@
       <c r="F27" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G27" s="7" t="n"/>
+      <c r="G27" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H27" s="7" t="n"/>
       <c r="I27" s="7" t="n"/>
       <c r="J27" s="7" t="n"/>
@@ -2755,7 +2807,9 @@
       <c r="F28" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G28" s="7" t="n"/>
+      <c r="G28" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H28" s="7" t="n"/>
       <c r="I28" s="7" t="n"/>
       <c r="J28" s="7" t="n"/>
@@ -2787,7 +2841,9 @@
       <c r="F29" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="7" t="n"/>
+      <c r="G29" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H29" s="7" t="n"/>
       <c r="I29" s="7" t="n"/>
       <c r="J29" s="7" t="n"/>
@@ -2819,7 +2875,9 @@
       <c r="F30" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G30" s="7" t="n"/>
+      <c r="G30" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H30" s="7" t="n"/>
       <c r="I30" s="7" t="n"/>
       <c r="J30" s="7" t="n"/>
@@ -2851,7 +2909,9 @@
       <c r="F31" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G31" s="7" t="n"/>
+      <c r="G31" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="H31" s="7" t="n"/>
       <c r="I31" s="7" t="n"/>
       <c r="J31" s="7" t="n"/>
@@ -2883,7 +2943,9 @@
       <c r="F32" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G32" s="7" t="n"/>
+      <c r="G32" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H32" s="7" t="n"/>
       <c r="I32" s="7" t="n"/>
       <c r="J32" s="7" t="n"/>
@@ -2915,7 +2977,9 @@
       <c r="F33" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G33" s="7" t="n"/>
+      <c r="G33" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="H33" s="7" t="n"/>
       <c r="I33" s="7" t="n"/>
       <c r="J33" s="7" t="n"/>
@@ -2947,7 +3011,9 @@
       <c r="F34" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G34" s="7" t="n"/>
+      <c r="G34" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="H34" s="7" t="n"/>
       <c r="I34" s="7" t="n"/>
       <c r="J34" s="7" t="n"/>

</xml_diff>

<commit_message>
Stats bijgewerkt t/m 10-10-2026 (telefoon): 4-4 tegen De Merino's 2, Jelmer nieuw in selectie
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015WZFvXLYMKyAxjcVaLguDM
</commit_message>
<xml_diff>
--- a/data/WB3 Stats.xlsx
+++ b/data/WB3 Stats.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Selectie" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Training" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Competitie" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Oefen" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Wedstrijden" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selectie" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitie" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oefen" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wedstrijden" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Selectie'!$A$2:$N$35</definedName>
@@ -1595,15 +1595,28 @@
       <c r="N35" s="7" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="n"/>
-      <c r="B36" s="7" t="n"/>
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>Jelmer</t>
+        </is>
+      </c>
+      <c r="B36" s="7">
+        <f>SUM(Competitie!B35:Q35)</f>
+        <v/>
+      </c>
       <c r="C36" s="7" t="n"/>
       <c r="D36" s="7" t="n"/>
       <c r="E36" s="7" t="n"/>
       <c r="F36" s="7" t="n"/>
       <c r="G36" s="7" t="n"/>
-      <c r="H36" s="7" t="n"/>
-      <c r="I36" s="7" t="n"/>
+      <c r="H36" s="7">
+        <f>SUM(Training!B35:P35)</f>
+        <v/>
+      </c>
+      <c r="I36" s="7">
+        <f>SUM(Oefen!B35:O35)</f>
+        <v/>
+      </c>
       <c r="J36" s="7" t="n"/>
       <c r="K36" s="7" t="n"/>
       <c r="L36" s="7" t="n"/>
@@ -3025,7 +3038,11 @@
       <c r="P34" s="7" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="n"/>
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Jelmer</t>
+        </is>
+      </c>
       <c r="B35" s="7" t="n"/>
       <c r="C35" s="7" t="n"/>
       <c r="D35" s="7" t="n"/>
@@ -4338,7 +4355,11 @@
       <c r="Q34" s="7" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="n"/>
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Jelmer</t>
+        </is>
+      </c>
       <c r="B35" s="7" t="n"/>
       <c r="C35" s="7" t="n"/>
       <c r="D35" s="7" t="n"/>
@@ -5427,7 +5448,11 @@
       <c r="Q34" s="7" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="n"/>
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Jelmer</t>
+        </is>
+      </c>
       <c r="B35" s="7" t="n"/>
       <c r="C35" s="7" t="n"/>
       <c r="D35" s="7" t="n"/>

</xml_diff>

<commit_message>
Stats bijgewerkt t/m 20 oktober (WB3 - Woudenberg 2 3-1)
Oefenpot tegen het tweede, training 15 oktober, Ricardo nieuw.
build.py: 'van' = 'v.' in namen, Stats-regel zonder dubbele punt
wordt alsnog herkend. Opmerking bij de wedstrijd toegevoegd.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/WB3 Stats.xlsx
+++ b/data/WB3 Stats.xlsx
@@ -10,8 +10,8 @@
     <sheet name="Wedstrijden" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Selectie'!$A$2:$N$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Training'!$A$1:$P$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Selectie'!$A$2:$N$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Training'!$A$1:$P$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N47"/>
+  <dimension ref="A1:N48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.880000000000001" customWidth="1" style="15" min="2" max="2"/>
@@ -634,7 +634,7 @@
         <v/>
       </c>
       <c r="I4" s="7">
-        <f>SUM(Oefen!B4:O4)</f>
+        <f>SUM(Oefen!B3:O3)</f>
         <v/>
       </c>
       <c r="J4" s="7" t="n"/>
@@ -663,7 +663,7 @@
         <v/>
       </c>
       <c r="I5" s="7">
-        <f>SUM(Oefen!B5:O5)</f>
+        <f>SUM(Oefen!B4:O4)</f>
         <v/>
       </c>
       <c r="J5" s="7" t="n"/>
@@ -1098,7 +1098,9 @@
       <c r="K19" s="7" t="n"/>
       <c r="L19" s="7" t="n"/>
       <c r="M19" s="7" t="n"/>
-      <c r="N19" s="7" t="n"/>
+      <c r="N19" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1222,10 +1224,13 @@
         <f>SUM(Training!B22:P22)</f>
         <v/>
       </c>
-      <c r="I23" s="7" t="n">
-        <v>90</v>
-      </c>
-      <c r="J23" s="7" t="n"/>
+      <c r="I23" s="7">
+        <f>SUM(Oefen!B22:O22)</f>
+        <v/>
+      </c>
+      <c r="J23" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="K23" s="7" t="n">
         <v>2</v>
       </c>
@@ -1255,7 +1260,7 @@
         <v/>
       </c>
       <c r="I24" s="7">
-        <f>SUM(Oefen!B24:O24)</f>
+        <f>SUM(Oefen!B23:O23)</f>
         <v/>
       </c>
       <c r="J24" s="7" t="n"/>
@@ -1288,7 +1293,7 @@
         <v/>
       </c>
       <c r="I25" s="7">
-        <f>SUM(Oefen!B25:O25)</f>
+        <f>SUM(Oefen!B24:O24)</f>
         <v/>
       </c>
       <c r="J25" s="7" t="n"/>
@@ -1321,7 +1326,7 @@
         <v/>
       </c>
       <c r="I26" s="7">
-        <f>SUM(Oefen!B26:O26)</f>
+        <f>SUM(Oefen!B25:O25)</f>
         <v/>
       </c>
       <c r="J26" s="7" t="n"/>
@@ -1350,7 +1355,7 @@
         <v/>
       </c>
       <c r="I27" s="7">
-        <f>SUM(Oefen!B27:O27)</f>
+        <f>SUM(Oefen!B26:O26)</f>
         <v/>
       </c>
       <c r="J27" s="7" t="n"/>
@@ -1379,7 +1384,7 @@
         <v/>
       </c>
       <c r="I28" s="7">
-        <f>SUM(Oefen!B28:O28)</f>
+        <f>SUM(Oefen!B27:O27)</f>
         <v/>
       </c>
       <c r="J28" s="7" t="n">
@@ -1410,11 +1415,13 @@
         <v/>
       </c>
       <c r="I29" s="7">
-        <f>SUM(Oefen!B29:O29)</f>
+        <f>SUM(Oefen!B28:O28)</f>
         <v/>
       </c>
       <c r="J29" s="7" t="n"/>
-      <c r="K29" s="7" t="n"/>
+      <c r="K29" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="L29" s="7" t="n"/>
       <c r="M29" s="7" t="n"/>
       <c r="N29" s="7" t="n"/>
@@ -1422,11 +1429,11 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Robert H.</t>
+          <t>Ricardo</t>
         </is>
       </c>
       <c r="B30" s="7">
-        <f>SUM(Competitie!B29:Q29)</f>
+        <f>SUM(Competitie!B30:Q30)</f>
         <v/>
       </c>
       <c r="C30" s="7" t="n"/>
@@ -1435,11 +1442,11 @@
       <c r="F30" s="7" t="n"/>
       <c r="G30" s="7" t="n"/>
       <c r="H30" s="7">
-        <f>SUM(Training!B29:P29)</f>
+        <f>SUM(Training!B30:P30)</f>
         <v/>
       </c>
       <c r="I30" s="7">
-        <f>SUM(Oefen!B30:O30)</f>
+        <f>SUM(Oefen!B29:O29)</f>
         <v/>
       </c>
       <c r="J30" s="7" t="n"/>
@@ -1451,7 +1458,7 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Robin v. B.</t>
+          <t>Robert H.</t>
         </is>
       </c>
       <c r="B31" s="7">
@@ -1468,7 +1475,7 @@
         <v/>
       </c>
       <c r="I31" s="7">
-        <f>SUM(Oefen!B31:O31)</f>
+        <f>SUM(Oefen!B30:O30)</f>
         <v/>
       </c>
       <c r="J31" s="7" t="n"/>
@@ -1480,7 +1487,7 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Robin E.</t>
+          <t>Robin v. B.</t>
         </is>
       </c>
       <c r="B32" s="7">
@@ -1497,7 +1504,7 @@
         <v/>
       </c>
       <c r="I32" s="7">
-        <f>SUM(Oefen!B32:O32)</f>
+        <f>SUM(Oefen!B31:O31)</f>
         <v/>
       </c>
       <c r="J32" s="7" t="n"/>
@@ -1509,7 +1516,7 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Sander</t>
+          <t>Robin E.</t>
         </is>
       </c>
       <c r="B33" s="7">
@@ -1517,12 +1524,8 @@
         <v/>
       </c>
       <c r="C33" s="7" t="n"/>
-      <c r="D33" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="E33" s="7" t="n">
-        <v>1</v>
-      </c>
+      <c r="D33" s="7" t="n"/>
+      <c r="E33" s="7" t="n"/>
       <c r="F33" s="7" t="n"/>
       <c r="G33" s="7" t="n"/>
       <c r="H33" s="7">
@@ -1530,7 +1533,7 @@
         <v/>
       </c>
       <c r="I33" s="7">
-        <f>SUM(Oefen!B33:O33)</f>
+        <f>SUM(Oefen!B32:O32)</f>
         <v/>
       </c>
       <c r="J33" s="7" t="n"/>
@@ -1542,7 +1545,7 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Steven</t>
+          <t>Sander</t>
         </is>
       </c>
       <c r="B34" s="7">
@@ -1550,8 +1553,12 @@
         <v/>
       </c>
       <c r="C34" s="7" t="n"/>
-      <c r="D34" s="7" t="n"/>
-      <c r="E34" s="7" t="n"/>
+      <c r="D34" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E34" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F34" s="7" t="n"/>
       <c r="G34" s="7" t="n"/>
       <c r="H34" s="7">
@@ -1559,7 +1566,7 @@
         <v/>
       </c>
       <c r="I34" s="7">
-        <f>SUM(Oefen!B34:O34)</f>
+        <f>SUM(Oefen!B33:O33)</f>
         <v/>
       </c>
       <c r="J34" s="7" t="n"/>
@@ -1571,7 +1578,7 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Thijs</t>
+          <t>Steven</t>
         </is>
       </c>
       <c r="B35" s="7">
@@ -1588,7 +1595,7 @@
         <v/>
       </c>
       <c r="I35" s="7">
-        <f>SUM(Oefen!B35:O35)</f>
+        <f>SUM(Oefen!B34:O34)</f>
         <v/>
       </c>
       <c r="J35" s="7" t="n"/>
@@ -1600,30 +1607,24 @@
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>Tom</t>
+          <t>Thijs</t>
         </is>
       </c>
       <c r="B36" s="7">
         <f>SUM(Competitie!B35:Q35)</f>
         <v/>
       </c>
-      <c r="C36" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="D36" s="7" t="n">
-        <v>3</v>
-      </c>
+      <c r="C36" s="7" t="n"/>
+      <c r="D36" s="7" t="n"/>
       <c r="E36" s="7" t="n"/>
       <c r="F36" s="7" t="n"/>
-      <c r="G36" s="7" t="n">
-        <v>1</v>
-      </c>
+      <c r="G36" s="7" t="n"/>
       <c r="H36" s="7">
         <f>SUM(Training!B35:P35)</f>
         <v/>
       </c>
       <c r="I36" s="7">
-        <f>SUM(Oefen!B36:O36)</f>
+        <f>SUM(Oefen!B35:O35)</f>
         <v/>
       </c>
       <c r="J36" s="7" t="n"/>
@@ -1633,92 +1634,113 @@
       <c r="N36" s="7" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="n"/>
-      <c r="B37" s="7" t="n"/>
-      <c r="C37" s="7" t="n"/>
-      <c r="D37" s="7" t="n"/>
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>Tom</t>
+        </is>
+      </c>
+      <c r="B37" s="7">
+        <f>SUM(Competitie!B36:Q36)</f>
+        <v/>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>3</v>
+      </c>
       <c r="E37" s="7" t="n"/>
       <c r="F37" s="7" t="n"/>
-      <c r="G37" s="7" t="n"/>
-      <c r="H37" s="7" t="n"/>
-      <c r="I37" s="7" t="n"/>
-      <c r="J37" s="7" t="n"/>
+      <c r="G37" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" s="7">
+        <f>SUM(Training!B36:P36)</f>
+        <v/>
+      </c>
+      <c r="I37" s="7">
+        <f>SUM(Oefen!B36:O36)</f>
+        <v/>
+      </c>
+      <c r="J37" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="K37" s="7" t="n"/>
       <c r="L37" s="7" t="n"/>
       <c r="M37" s="7" t="n"/>
       <c r="N37" s="7" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="A38" s="7" t="n"/>
+      <c r="B38" s="7" t="n"/>
+      <c r="C38" s="7" t="n"/>
+      <c r="D38" s="7" t="n"/>
+      <c r="E38" s="7" t="n"/>
+      <c r="F38" s="7" t="n"/>
+      <c r="G38" s="7" t="n"/>
+      <c r="H38" s="7" t="n"/>
+      <c r="I38" s="7" t="n"/>
+      <c r="J38" s="7" t="n"/>
+      <c r="K38" s="7" t="n"/>
+      <c r="L38" s="7" t="n"/>
+      <c r="M38" s="7" t="n"/>
+      <c r="N38" s="7" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>Totaal</t>
         </is>
       </c>
-      <c r="B38" s="8">
-        <f>SUM(B3:B36)/990</f>
-        <v/>
-      </c>
-      <c r="C38" s="8">
-        <f>SUM(C3:C36)</f>
-        <v/>
-      </c>
-      <c r="D38" s="8">
-        <f>SUM(D3:D36)</f>
-        <v/>
-      </c>
-      <c r="E38" s="8">
-        <f>SUM(E3:E36)</f>
-        <v/>
-      </c>
-      <c r="F38" s="8">
-        <f>SUM(F3:F36)</f>
-        <v/>
-      </c>
-      <c r="G38" s="8">
-        <f>SUM(G3:G36)</f>
-        <v/>
-      </c>
-      <c r="H38" s="8" t="n"/>
-      <c r="I38" s="8">
-        <f>SUM(I3:I36)/990</f>
-        <v/>
-      </c>
-      <c r="J38" s="8">
-        <f>SUM(J3:J36)</f>
-        <v/>
-      </c>
-      <c r="K38" s="8">
-        <f>SUM(K3:K36)</f>
-        <v/>
-      </c>
-      <c r="L38" s="8">
-        <f>SUM(L3:L36)</f>
-        <v/>
-      </c>
-      <c r="M38" s="8">
-        <f>SUM(M3:M36)</f>
-        <v/>
-      </c>
-      <c r="N38" s="8">
-        <f>SUM(N3:N36)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="7" t="n"/>
-      <c r="B39" s="7" t="n"/>
-      <c r="C39" s="7" t="n"/>
-      <c r="D39" s="7" t="n"/>
-      <c r="E39" s="7" t="n"/>
-      <c r="F39" s="7" t="n"/>
-      <c r="G39" s="7" t="n"/>
-      <c r="H39" s="7" t="n"/>
-      <c r="I39" s="7" t="n"/>
-      <c r="J39" s="7" t="n"/>
-      <c r="K39" s="7" t="n"/>
-      <c r="L39" s="7" t="n"/>
-      <c r="M39" s="7" t="n"/>
-      <c r="N39" s="7" t="n"/>
+      <c r="B39" s="8">
+        <f>SUM(B3:B37)/990</f>
+        <v/>
+      </c>
+      <c r="C39" s="8">
+        <f>SUM(C3:C37)</f>
+        <v/>
+      </c>
+      <c r="D39" s="8">
+        <f>SUM(D3:D37)</f>
+        <v/>
+      </c>
+      <c r="E39" s="8">
+        <f>SUM(E3:E37)</f>
+        <v/>
+      </c>
+      <c r="F39" s="8">
+        <f>SUM(F3:F37)</f>
+        <v/>
+      </c>
+      <c r="G39" s="8">
+        <f>SUM(G3:G37)</f>
+        <v/>
+      </c>
+      <c r="H39" s="8" t="n"/>
+      <c r="I39" s="8">
+        <f>SUM(I3:I37)/990</f>
+        <v/>
+      </c>
+      <c r="J39" s="8">
+        <f>SUM(J3:J37)</f>
+        <v/>
+      </c>
+      <c r="K39" s="8">
+        <f>SUM(K3:K37)</f>
+        <v/>
+      </c>
+      <c r="L39" s="8">
+        <f>SUM(L3:L37)</f>
+        <v/>
+      </c>
+      <c r="M39" s="8">
+        <f>SUM(M3:M37)</f>
+        <v/>
+      </c>
+      <c r="N39" s="8">
+        <f>SUM(N3:N37)</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="n"/>
@@ -1848,8 +1870,24 @@
       <c r="M47" s="7" t="n"/>
       <c r="N47" s="7" t="n"/>
     </row>
+    <row r="48">
+      <c r="A48" s="7" t="n"/>
+      <c r="B48" s="7" t="n"/>
+      <c r="C48" s="7" t="n"/>
+      <c r="D48" s="7" t="n"/>
+      <c r="E48" s="7" t="n"/>
+      <c r="F48" s="7" t="n"/>
+      <c r="G48" s="7" t="n"/>
+      <c r="H48" s="7" t="n"/>
+      <c r="I48" s="7" t="n"/>
+      <c r="J48" s="7" t="n"/>
+      <c r="K48" s="7" t="n"/>
+      <c r="L48" s="7" t="n"/>
+      <c r="M48" s="7" t="n"/>
+      <c r="N48" s="7" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="$A$2:$N$36"/>
+  <autoFilter ref="$A$2:$N$37"/>
   <mergeCells count="2">
     <mergeCell ref="I1:N1"/>
     <mergeCell ref="B1:G1"/>
@@ -1864,7 +1902,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y49"/>
+  <dimension ref="A1:Y50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="8.880000000000001" customWidth="1" style="15" min="2" max="2"/>
@@ -2915,14 +2953,14 @@
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Robert H.</t>
+          <t>Ricardo</t>
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C29" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D29" s="7" t="n">
         <v>0</v>
@@ -2951,14 +2989,14 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Robin v. B.</t>
+          <t>Robert H.</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C30" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D30" s="7" t="n">
         <v>0</v>
@@ -2987,14 +3025,14 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Robin E.</t>
+          <t>Robin v. B.</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
         <v>0</v>
       </c>
       <c r="C31" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D31" s="7" t="n">
         <v>0</v>
@@ -3023,26 +3061,26 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Sander</t>
+          <t>Robin E.</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C32" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D32" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E32" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F32" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H32" s="7" t="n">
         <v>0</v>
@@ -3059,26 +3097,26 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Steven</t>
+          <t>Sander</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C33" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D33" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F33" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G33" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H33" s="7" t="n">
         <v>0</v>
@@ -3095,14 +3133,14 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Thijs</t>
+          <t>Steven</t>
         </is>
       </c>
       <c r="B34" s="7" t="n">
         <v>0</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D34" s="7" t="n">
         <v>0</v>
@@ -3111,7 +3149,7 @@
         <v>0</v>
       </c>
       <c r="F34" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G34" s="7" t="n">
         <v>0</v>
@@ -3131,14 +3169,14 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Tom</t>
+          <t>Thijs</t>
         </is>
       </c>
       <c r="B35" s="7" t="n">
         <v>0</v>
       </c>
       <c r="C35" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D35" s="7" t="n">
         <v>0</v>
@@ -3150,10 +3188,10 @@
         <v>0</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I35" s="7" t="n"/>
       <c r="J35" s="7" t="n"/>
@@ -3165,14 +3203,32 @@
       <c r="P35" s="7" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="n"/>
-      <c r="B36" s="7" t="n"/>
-      <c r="C36" s="7" t="n"/>
-      <c r="D36" s="7" t="n"/>
-      <c r="E36" s="7" t="n"/>
-      <c r="F36" s="7" t="n"/>
-      <c r="G36" s="7" t="n"/>
-      <c r="H36" s="7" t="n"/>
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>Tom</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="I36" s="7" t="n"/>
       <c r="J36" s="7" t="n"/>
       <c r="K36" s="7" t="n"/>
@@ -3183,39 +3239,14 @@
       <c r="P36" s="7" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="inlineStr">
-        <is>
-          <t>Totaal</t>
-        </is>
-      </c>
-      <c r="B37" s="8">
-        <f>SUM(B2:B35)</f>
-        <v/>
-      </c>
-      <c r="C37" s="8">
-        <f>SUM(C2:C35)</f>
-        <v/>
-      </c>
-      <c r="D37" s="8">
-        <f>SUM(D2:D35)</f>
-        <v/>
-      </c>
-      <c r="E37" s="8">
-        <f>SUM(E2:E35)</f>
-        <v/>
-      </c>
-      <c r="F37" s="8">
-        <f>SUM(F2:F35)</f>
-        <v/>
-      </c>
-      <c r="G37" s="8">
-        <f>SUM(G2:G35)</f>
-        <v/>
-      </c>
-      <c r="H37" s="8">
-        <f>SUM(H2:H35)</f>
-        <v/>
-      </c>
+      <c r="A37" s="7" t="n"/>
+      <c r="B37" s="7" t="n"/>
+      <c r="C37" s="7" t="n"/>
+      <c r="D37" s="7" t="n"/>
+      <c r="E37" s="7" t="n"/>
+      <c r="F37" s="7" t="n"/>
+      <c r="G37" s="7" t="n"/>
+      <c r="H37" s="7" t="n"/>
       <c r="I37" s="7" t="n"/>
       <c r="J37" s="7" t="n"/>
       <c r="K37" s="7" t="n"/>
@@ -3226,14 +3257,39 @@
       <c r="P37" s="7" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="n"/>
-      <c r="B38" s="7" t="n"/>
-      <c r="C38" s="7" t="n"/>
-      <c r="D38" s="7" t="n"/>
-      <c r="E38" s="7" t="n"/>
-      <c r="F38" s="7" t="n"/>
-      <c r="G38" s="8" t="n"/>
-      <c r="H38" s="7" t="n"/>
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Totaal</t>
+        </is>
+      </c>
+      <c r="B38" s="8">
+        <f>SUM(B2:B36)</f>
+        <v/>
+      </c>
+      <c r="C38" s="8">
+        <f>SUM(C2:C36)</f>
+        <v/>
+      </c>
+      <c r="D38" s="8">
+        <f>SUM(D2:D36)</f>
+        <v/>
+      </c>
+      <c r="E38" s="8">
+        <f>SUM(E2:E36)</f>
+        <v/>
+      </c>
+      <c r="F38" s="8">
+        <f>SUM(F2:F36)</f>
+        <v/>
+      </c>
+      <c r="G38" s="8">
+        <f>SUM(G2:G36)</f>
+        <v/>
+      </c>
+      <c r="H38" s="8">
+        <f>SUM(H2:H36)</f>
+        <v/>
+      </c>
       <c r="I38" s="7" t="n"/>
       <c r="J38" s="7" t="n"/>
       <c r="K38" s="7" t="n"/>
@@ -3250,7 +3306,7 @@
       <c r="D39" s="7" t="n"/>
       <c r="E39" s="7" t="n"/>
       <c r="F39" s="7" t="n"/>
-      <c r="G39" s="7" t="n"/>
+      <c r="G39" s="8" t="n"/>
       <c r="H39" s="7" t="n"/>
       <c r="I39" s="7" t="n"/>
       <c r="J39" s="7" t="n"/>
@@ -3441,13 +3497,31 @@
       <c r="O49" s="7" t="n"/>
       <c r="P49" s="7" t="n"/>
     </row>
+    <row r="50">
+      <c r="A50" s="7" t="n"/>
+      <c r="B50" s="7" t="n"/>
+      <c r="C50" s="7" t="n"/>
+      <c r="D50" s="7" t="n"/>
+      <c r="E50" s="7" t="n"/>
+      <c r="F50" s="7" t="n"/>
+      <c r="G50" s="7" t="n"/>
+      <c r="H50" s="7" t="n"/>
+      <c r="I50" s="7" t="n"/>
+      <c r="J50" s="7" t="n"/>
+      <c r="K50" s="7" t="n"/>
+      <c r="L50" s="7" t="n"/>
+      <c r="M50" s="7" t="n"/>
+      <c r="N50" s="7" t="n"/>
+      <c r="O50" s="7" t="n"/>
+      <c r="P50" s="7" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="$A$1:$P$35">
-    <sortState ref="A1:P35">
-      <sortCondition ref="A1:A35"/>
+  <autoFilter ref="$A$1:$P$36">
+    <sortState ref="A1:P36">
+      <sortCondition ref="A1:A36"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="B1:P1019">
+  <conditionalFormatting sqref="B1:P1020">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>1</formula>
     </cfRule>
@@ -3465,7 +3539,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q46"/>
+  <dimension ref="A1:Q47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="6.25" customWidth="1" style="15" min="2" max="17"/>
@@ -4366,7 +4440,7 @@
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Robert H.</t>
+          <t>Ricardo</t>
         </is>
       </c>
       <c r="B29" s="7" t="n">
@@ -4397,20 +4471,20 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Robin v. B.</t>
+          <t>Robert H.</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
         <v>0</v>
       </c>
       <c r="C30" s="7" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="D30" s="7" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="F30" s="7" t="n"/>
       <c r="G30" s="7" t="n"/>
@@ -4428,20 +4502,20 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Robin E.</t>
+          <t>Robin v. B.</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
         <v>0</v>
       </c>
       <c r="C31" s="7" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="D31" s="7" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F31" s="7" t="n"/>
       <c r="G31" s="7" t="n"/>
@@ -4459,20 +4533,20 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Sander</t>
+          <t>Robin E.</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="C32" s="7" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="D32" s="7" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="E32" s="7" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="F32" s="7" t="n"/>
       <c r="G32" s="7" t="n"/>
@@ -4490,20 +4564,20 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Steven</t>
+          <t>Sander</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="C33" s="7" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="D33" s="7" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F33" s="7" t="n"/>
       <c r="G33" s="7" t="n"/>
@@ -4521,14 +4595,14 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Thijs</t>
+          <t>Steven</t>
         </is>
       </c>
       <c r="B34" s="7" t="n">
         <v>0</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="D34" s="7" t="n">
         <v>0</v>
@@ -4552,20 +4626,20 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Tom</t>
+          <t>Thijs</t>
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="C35" s="7" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="D35" s="7" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="F35" s="7" t="n"/>
       <c r="G35" s="7" t="n"/>
@@ -4581,11 +4655,23 @@
       <c r="Q35" s="7" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="n"/>
-      <c r="B36" s="7" t="n"/>
-      <c r="C36" s="7" t="n"/>
-      <c r="D36" s="7" t="n"/>
-      <c r="E36" s="7" t="n"/>
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>Tom</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>90</v>
+      </c>
       <c r="F36" s="7" t="n"/>
       <c r="G36" s="7" t="n"/>
       <c r="H36" s="7" t="n"/>
@@ -4600,28 +4686,12 @@
       <c r="Q36" s="7" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="inlineStr">
-        <is>
-          <t>Totaal</t>
-        </is>
-      </c>
-      <c r="B37" s="8">
-        <f>SUM(B2:B35)</f>
-        <v/>
-      </c>
-      <c r="C37" s="8">
-        <f>SUM(C2:C35)</f>
-        <v/>
-      </c>
-      <c r="D37" s="8">
-        <f>SUM(D2:D35)</f>
-        <v/>
-      </c>
-      <c r="E37" s="8">
-        <f>SUM(E2:E35)</f>
-        <v/>
-      </c>
-      <c r="F37" s="8" t="n"/>
+      <c r="A37" s="7" t="n"/>
+      <c r="B37" s="7" t="n"/>
+      <c r="C37" s="7" t="n"/>
+      <c r="D37" s="7" t="n"/>
+      <c r="E37" s="7" t="n"/>
+      <c r="F37" s="7" t="n"/>
       <c r="G37" s="7" t="n"/>
       <c r="H37" s="7" t="n"/>
       <c r="I37" s="7" t="n"/>
@@ -4635,12 +4705,28 @@
       <c r="Q37" s="7" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="n"/>
-      <c r="B38" s="7" t="n"/>
-      <c r="C38" s="7" t="n"/>
-      <c r="D38" s="7" t="n"/>
-      <c r="E38" s="7" t="n"/>
-      <c r="F38" s="7" t="n"/>
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Totaal</t>
+        </is>
+      </c>
+      <c r="B38" s="8">
+        <f>SUM(B2:B36)</f>
+        <v/>
+      </c>
+      <c r="C38" s="8">
+        <f>SUM(C2:C36)</f>
+        <v/>
+      </c>
+      <c r="D38" s="8">
+        <f>SUM(D2:D36)</f>
+        <v/>
+      </c>
+      <c r="E38" s="8">
+        <f>SUM(E2:E36)</f>
+        <v/>
+      </c>
+      <c r="F38" s="8" t="n"/>
       <c r="G38" s="7" t="n"/>
       <c r="H38" s="7" t="n"/>
       <c r="I38" s="7" t="n"/>
@@ -4805,6 +4891,25 @@
       <c r="P46" s="7" t="n"/>
       <c r="Q46" s="7" t="n"/>
     </row>
+    <row r="47">
+      <c r="A47" s="7" t="n"/>
+      <c r="B47" s="7" t="n"/>
+      <c r="C47" s="7" t="n"/>
+      <c r="D47" s="7" t="n"/>
+      <c r="E47" s="7" t="n"/>
+      <c r="F47" s="7" t="n"/>
+      <c r="G47" s="7" t="n"/>
+      <c r="H47" s="7" t="n"/>
+      <c r="I47" s="7" t="n"/>
+      <c r="J47" s="7" t="n"/>
+      <c r="K47" s="7" t="n"/>
+      <c r="L47" s="7" t="n"/>
+      <c r="M47" s="7" t="n"/>
+      <c r="N47" s="7" t="n"/>
+      <c r="O47" s="7" t="n"/>
+      <c r="P47" s="7" t="n"/>
+      <c r="Q47" s="7" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4816,7 +4921,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q46"/>
+  <dimension ref="A1:Q47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="6.25" customWidth="1" style="15" min="2" max="17"/>
@@ -4831,7 +4936,9 @@
       <c r="B1" s="9" t="n">
         <v>46274</v>
       </c>
-      <c r="C1" s="9" t="n"/>
+      <c r="C1" s="9" t="n">
+        <v>46315</v>
+      </c>
       <c r="D1" s="9" t="n"/>
       <c r="E1" s="9" t="n"/>
       <c r="F1" s="9" t="n"/>
@@ -4856,7 +4963,9 @@
       <c r="B2" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C2" s="7" t="n"/>
+      <c r="C2" s="7" t="n">
+        <v>30</v>
+      </c>
       <c r="D2" s="7" t="n"/>
       <c r="E2" s="7" t="n"/>
       <c r="F2" s="7" t="n"/>
@@ -4881,7 +4990,9 @@
       <c r="B3" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C3" s="7" t="n"/>
+      <c r="C3" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D3" s="7" t="n"/>
       <c r="E3" s="7" t="n"/>
       <c r="F3" s="7" t="n"/>
@@ -4906,7 +5017,9 @@
       <c r="B4" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="7" t="n"/>
+      <c r="C4" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D4" s="7" t="n"/>
       <c r="E4" s="7" t="n"/>
       <c r="F4" s="7" t="n"/>
@@ -4931,7 +5044,9 @@
       <c r="B5" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="7" t="n"/>
+      <c r="C5" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D5" s="7" t="n"/>
       <c r="E5" s="7" t="n"/>
       <c r="F5" s="7" t="n"/>
@@ -4956,7 +5071,9 @@
       <c r="B6" s="7" t="n">
         <v>45</v>
       </c>
-      <c r="C6" s="7" t="n"/>
+      <c r="C6" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D6" s="7" t="n"/>
       <c r="E6" s="7" t="n"/>
       <c r="F6" s="7" t="n"/>
@@ -4981,7 +5098,9 @@
       <c r="B7" s="7" t="n">
         <v>90</v>
       </c>
-      <c r="C7" s="7" t="n"/>
+      <c r="C7" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D7" s="7" t="n"/>
       <c r="E7" s="7" t="n"/>
       <c r="F7" s="7" t="n"/>
@@ -5006,7 +5125,9 @@
       <c r="B8" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C8" s="7" t="n"/>
+      <c r="C8" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D8" s="7" t="n"/>
       <c r="E8" s="7" t="n"/>
       <c r="F8" s="7" t="n"/>
@@ -5031,7 +5152,9 @@
       <c r="B9" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="7" t="n"/>
+      <c r="C9" s="7" t="n">
+        <v>90</v>
+      </c>
       <c r="D9" s="7" t="n"/>
       <c r="E9" s="7" t="n"/>
       <c r="F9" s="7" t="n"/>
@@ -5056,7 +5179,9 @@
       <c r="B10" s="7" t="n">
         <v>45</v>
       </c>
-      <c r="C10" s="7" t="n"/>
+      <c r="C10" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D10" s="7" t="n"/>
       <c r="E10" s="7" t="n"/>
       <c r="F10" s="7" t="n"/>
@@ -5081,7 +5206,9 @@
       <c r="B11" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="C11" s="7" t="n"/>
+      <c r="C11" s="7" t="n">
+        <v>45</v>
+      </c>
       <c r="D11" s="7" t="n"/>
       <c r="E11" s="7" t="n"/>
       <c r="F11" s="7" t="n"/>
@@ -5106,7 +5233,9 @@
       <c r="B12" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C12" s="7" t="n"/>
+      <c r="C12" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D12" s="7" t="n"/>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="7" t="n"/>
@@ -5131,7 +5260,9 @@
       <c r="B13" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C13" s="7" t="n"/>
+      <c r="C13" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D13" s="7" t="n"/>
       <c r="E13" s="7" t="n"/>
       <c r="F13" s="7" t="n"/>
@@ -5156,7 +5287,9 @@
       <c r="B14" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C14" s="7" t="n"/>
+      <c r="C14" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D14" s="7" t="n"/>
       <c r="E14" s="7" t="n"/>
       <c r="F14" s="7" t="n"/>
@@ -5181,7 +5314,9 @@
       <c r="B15" s="7" t="n">
         <v>45</v>
       </c>
-      <c r="C15" s="7" t="n"/>
+      <c r="C15" s="7" t="n">
+        <v>90</v>
+      </c>
       <c r="D15" s="7" t="n"/>
       <c r="E15" s="7" t="n"/>
       <c r="F15" s="7" t="n"/>
@@ -5206,7 +5341,9 @@
       <c r="B16" s="7" t="n">
         <v>45</v>
       </c>
-      <c r="C16" s="7" t="n"/>
+      <c r="C16" s="7" t="n">
+        <v>90</v>
+      </c>
       <c r="D16" s="7" t="n"/>
       <c r="E16" s="7" t="n"/>
       <c r="F16" s="7" t="n"/>
@@ -5231,7 +5368,9 @@
       <c r="B17" s="7" t="n">
         <v>90</v>
       </c>
-      <c r="C17" s="7" t="n"/>
+      <c r="C17" s="7" t="n">
+        <v>45</v>
+      </c>
       <c r="D17" s="7" t="n"/>
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="7" t="n"/>
@@ -5256,7 +5395,9 @@
       <c r="B18" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C18" s="7" t="n"/>
+      <c r="C18" s="7" t="n">
+        <v>90</v>
+      </c>
       <c r="D18" s="7" t="n"/>
       <c r="E18" s="7" t="n"/>
       <c r="F18" s="7" t="n"/>
@@ -5281,7 +5422,9 @@
       <c r="B19" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C19" s="7" t="n"/>
+      <c r="C19" s="7" t="n">
+        <v>90</v>
+      </c>
       <c r="D19" s="7" t="n"/>
       <c r="E19" s="7" t="n"/>
       <c r="F19" s="7" t="n"/>
@@ -5306,7 +5449,9 @@
       <c r="B20" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="C20" s="7" t="n"/>
+      <c r="C20" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D20" s="7" t="n"/>
       <c r="E20" s="7" t="n"/>
       <c r="F20" s="7" t="n"/>
@@ -5331,7 +5476,9 @@
       <c r="B21" s="7" t="n">
         <v>90</v>
       </c>
-      <c r="C21" s="7" t="n"/>
+      <c r="C21" s="7" t="n">
+        <v>45</v>
+      </c>
       <c r="D21" s="7" t="n"/>
       <c r="E21" s="7" t="n"/>
       <c r="F21" s="7" t="n"/>
@@ -5356,7 +5503,9 @@
       <c r="B22" s="7" t="n">
         <v>90</v>
       </c>
-      <c r="C22" s="7" t="n"/>
+      <c r="C22" s="7" t="n">
+        <v>45</v>
+      </c>
       <c r="D22" s="7" t="n"/>
       <c r="E22" s="7" t="n"/>
       <c r="F22" s="7" t="n"/>
@@ -5381,7 +5530,9 @@
       <c r="B23" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C23" s="7" t="n"/>
+      <c r="C23" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D23" s="7" t="n"/>
       <c r="E23" s="7" t="n"/>
       <c r="F23" s="7" t="n"/>
@@ -5406,7 +5557,9 @@
       <c r="B24" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C24" s="7" t="n"/>
+      <c r="C24" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D24" s="7" t="n"/>
       <c r="E24" s="7" t="n"/>
       <c r="F24" s="7" t="n"/>
@@ -5431,7 +5584,9 @@
       <c r="B25" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C25" s="7" t="n"/>
+      <c r="C25" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D25" s="7" t="n"/>
       <c r="E25" s="7" t="n"/>
       <c r="F25" s="7" t="n"/>
@@ -5456,7 +5611,9 @@
       <c r="B26" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C26" s="7" t="n"/>
+      <c r="C26" s="7" t="n">
+        <v>45</v>
+      </c>
       <c r="D26" s="7" t="n"/>
       <c r="E26" s="7" t="n"/>
       <c r="F26" s="7" t="n"/>
@@ -5481,7 +5638,9 @@
       <c r="B27" s="7" t="n">
         <v>45</v>
       </c>
-      <c r="C27" s="7" t="n"/>
+      <c r="C27" s="7" t="n">
+        <v>45</v>
+      </c>
       <c r="D27" s="7" t="n"/>
       <c r="E27" s="7" t="n"/>
       <c r="F27" s="7" t="n"/>
@@ -5506,7 +5665,9 @@
       <c r="B28" s="7" t="n">
         <v>90</v>
       </c>
-      <c r="C28" s="7" t="n"/>
+      <c r="C28" s="7" t="n">
+        <v>90</v>
+      </c>
       <c r="D28" s="7" t="n"/>
       <c r="E28" s="7" t="n"/>
       <c r="F28" s="7" t="n"/>
@@ -5525,13 +5686,15 @@
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Robert H.</t>
+          <t>Ricardo</t>
         </is>
       </c>
       <c r="B29" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C29" s="7" t="n"/>
+      <c r="C29" s="7" t="n">
+        <v>90</v>
+      </c>
       <c r="D29" s="7" t="n"/>
       <c r="E29" s="7" t="n"/>
       <c r="F29" s="7" t="n"/>
@@ -5550,13 +5713,15 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Robin v. B.</t>
+          <t>Robert H.</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>90</v>
-      </c>
-      <c r="C30" s="7" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D30" s="7" t="n"/>
       <c r="E30" s="7" t="n"/>
       <c r="F30" s="7" t="n"/>
@@ -5575,13 +5740,15 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Robin E.</t>
+          <t>Robin v. B.</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C31" s="7" t="n"/>
+        <v>90</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D31" s="7" t="n"/>
       <c r="E31" s="7" t="n"/>
       <c r="F31" s="7" t="n"/>
@@ -5600,13 +5767,15 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Sander</t>
+          <t>Robin E.</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>90</v>
-      </c>
-      <c r="C32" s="7" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D32" s="7" t="n"/>
       <c r="E32" s="7" t="n"/>
       <c r="F32" s="7" t="n"/>
@@ -5625,13 +5794,15 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Steven</t>
+          <t>Sander</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="C33" s="7" t="n"/>
+        <v>90</v>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D33" s="7" t="n"/>
       <c r="E33" s="7" t="n"/>
       <c r="F33" s="7" t="n"/>
@@ -5650,13 +5821,15 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Thijs</t>
+          <t>Steven</t>
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C34" s="7" t="n"/>
+        <v>45</v>
+      </c>
+      <c r="C34" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D34" s="7" t="n"/>
       <c r="E34" s="7" t="n"/>
       <c r="F34" s="7" t="n"/>
@@ -5675,13 +5848,15 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Tom</t>
+          <t>Thijs</t>
         </is>
       </c>
       <c r="B35" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C35" s="7" t="n"/>
+      <c r="C35" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="D35" s="7" t="n"/>
       <c r="E35" s="7" t="n"/>
       <c r="F35" s="7" t="n"/>
@@ -5698,9 +5873,17 @@
       <c r="Q35" s="7" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="n"/>
-      <c r="B36" s="7" t="n"/>
-      <c r="C36" s="7" t="n"/>
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>Tom</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>60</v>
+      </c>
       <c r="D36" s="7" t="n"/>
       <c r="E36" s="7" t="n"/>
       <c r="F36" s="7" t="n"/>
@@ -5737,8 +5920,14 @@
     </row>
     <row r="38">
       <c r="A38" s="7" t="n"/>
-      <c r="B38" s="7" t="n"/>
-      <c r="C38" s="7" t="n"/>
+      <c r="B38" s="7">
+        <f>SUM(B2:B36)</f>
+        <v/>
+      </c>
+      <c r="C38" s="7">
+        <f>SUM(C2:C36)</f>
+        <v/>
+      </c>
       <c r="D38" s="7" t="n"/>
       <c r="E38" s="7" t="n"/>
       <c r="F38" s="7" t="n"/>
@@ -5906,6 +6095,25 @@
       <c r="P46" s="7" t="n"/>
       <c r="Q46" s="7" t="n"/>
     </row>
+    <row r="47">
+      <c r="A47" s="7" t="n"/>
+      <c r="B47" s="7" t="n"/>
+      <c r="C47" s="7" t="n"/>
+      <c r="D47" s="7" t="n"/>
+      <c r="E47" s="7" t="n"/>
+      <c r="F47" s="7" t="n"/>
+      <c r="G47" s="7" t="n"/>
+      <c r="H47" s="7" t="n"/>
+      <c r="I47" s="7" t="n"/>
+      <c r="J47" s="7" t="n"/>
+      <c r="K47" s="7" t="n"/>
+      <c r="L47" s="7" t="n"/>
+      <c r="M47" s="7" t="n"/>
+      <c r="N47" s="7" t="n"/>
+      <c r="O47" s="7" t="n"/>
+      <c r="P47" s="7" t="n"/>
+      <c r="Q47" s="7" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5917,7 +6125,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB27"/>
+  <dimension ref="A1:AB28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="10.75" customWidth="1" style="15" min="1" max="1"/>
@@ -6121,7 +6329,7 @@
       <c r="F5" s="7" t="inlineStr">
         <is>
           <t>Doelpunten: Tom 5x, Robin H. 1x
-Assists: Sander 2x, Jur, Niels v. B., Tom
+Assists: Sander 2x, Jur, Niels van B., Tom
 Snuiter: Tom</t>
         </is>
       </c>
@@ -6170,36 +6378,54 @@
     </row>
     <row r="7">
       <c r="A7" s="12" t="n">
-        <v>46319.58333333334</v>
-      </c>
-      <c r="B7" s="7" t="n"/>
+        <v>46315.83333333334</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Oefen</t>
+        </is>
+      </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>GVVV 2</t>
+          <t>Woudenberg 2</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Uit</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
-      <c r="G7" s="14" t="n"/>
+          <t>Thuis</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>3-1 (W)</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Doelpunten: Tom 2x, Mark
+Assists: Peter
+Snuiter Jur</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>Het tweede kwam met snelheid, conditie en een toekomst. Wij kwamen met ervaring, tape en een warming-up van tien minuten. Eindstand: opa's 3, kleinzoons 1. Jongens, het komt goed met jullie. Ooit.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="n">
-        <v>46326.625</v>
+        <v>46319.58333333334</v>
       </c>
       <c r="B8" s="7" t="n"/>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>VRC 2</t>
+          <t>GVVV 2</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Thuis</t>
+          <t>Uit</t>
         </is>
       </c>
       <c r="E8" s="7" t="n"/>
@@ -6208,17 +6434,17 @@
     </row>
     <row r="9">
       <c r="A9" s="12" t="n">
-        <v>46333.5</v>
+        <v>46326.625</v>
       </c>
       <c r="B9" s="7" t="n"/>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Renswoude 2</t>
+          <t>VRC 2</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Uit</t>
+          <t>Thuis</t>
         </is>
       </c>
       <c r="E9" s="7" t="n"/>
@@ -6227,17 +6453,17 @@
     </row>
     <row r="10">
       <c r="A10" s="12" t="n">
-        <v>46347.625</v>
+        <v>46333.5</v>
       </c>
       <c r="B10" s="7" t="n"/>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Candia '66 2</t>
+          <t>Renswoude 2</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Thuis</t>
+          <t>Uit</t>
         </is>
       </c>
       <c r="E10" s="7" t="n"/>
@@ -6246,17 +6472,17 @@
     </row>
     <row r="11">
       <c r="A11" s="12" t="n">
-        <v>46354.625</v>
+        <v>46347.625</v>
       </c>
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Roda '46 3</t>
+          <t>Candia '66 2</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Uit</t>
+          <t>Thuis</t>
         </is>
       </c>
       <c r="E11" s="7" t="n"/>
@@ -6265,17 +6491,17 @@
     </row>
     <row r="12">
       <c r="A12" s="12" t="n">
-        <v>46361.60416666666</v>
+        <v>46354.625</v>
       </c>
       <c r="B12" s="7" t="n"/>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>SVL 2</t>
+          <t>Roda '46 3</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Thuis</t>
+          <t>Uit</t>
         </is>
       </c>
       <c r="E12" s="7" t="n"/>
@@ -6284,12 +6510,12 @@
     </row>
     <row r="13">
       <c r="A13" s="12" t="n">
-        <v>46417.625</v>
+        <v>46361.60416666666</v>
       </c>
       <c r="B13" s="7" t="n"/>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>VVZA 2</t>
+          <t>SVL 2</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -6303,17 +6529,17 @@
     </row>
     <row r="14">
       <c r="A14" s="12" t="n">
-        <v>46424.5</v>
+        <v>46417.625</v>
       </c>
       <c r="B14" s="7" t="n"/>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>CDW 2</t>
+          <t>VVZA 2</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Uit</t>
+          <t>Thuis</t>
         </is>
       </c>
       <c r="E14" s="7" t="n"/>
@@ -6322,12 +6548,12 @@
     </row>
     <row r="15">
       <c r="A15" s="12" t="n">
-        <v>46445.60416666666</v>
+        <v>46424.5</v>
       </c>
       <c r="B15" s="7" t="n"/>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Valleivogels 3</t>
+          <t>CDW 2</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -6341,17 +6567,17 @@
     </row>
     <row r="16">
       <c r="A16" s="12" t="n">
-        <v>46452.625</v>
+        <v>46445.60416666666</v>
       </c>
       <c r="B16" s="7" t="n"/>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Hooglanderveen 2</t>
+          <t>Valleivogels 3</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Thuis</t>
+          <t>Uit</t>
         </is>
       </c>
       <c r="E16" s="7" t="n"/>
@@ -6360,17 +6586,17 @@
     </row>
     <row r="17">
       <c r="A17" s="12" t="n">
-        <v>46459.48958333334</v>
+        <v>46452.625</v>
       </c>
       <c r="B17" s="7" t="n"/>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>De Merino's 2</t>
+          <t>Hooglanderveen 2</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Uit</t>
+          <t>Thuis</t>
         </is>
       </c>
       <c r="E17" s="7" t="n"/>
@@ -6379,17 +6605,17 @@
     </row>
     <row r="18">
       <c r="A18" s="12" t="n">
-        <v>46466.625</v>
+        <v>46459.48958333334</v>
       </c>
       <c r="B18" s="7" t="n"/>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>GVVV 2</t>
+          <t>De Merino's 2</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Thuis</t>
+          <t>Uit</t>
         </is>
       </c>
       <c r="E18" s="7" t="n"/>
@@ -6398,17 +6624,17 @@
     </row>
     <row r="19">
       <c r="A19" s="12" t="n">
-        <v>46480.52083333334</v>
+        <v>46466.625</v>
       </c>
       <c r="B19" s="7" t="n"/>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>VRC 2</t>
+          <t>GVVV 2</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Uit</t>
+          <t>Thuis</t>
         </is>
       </c>
       <c r="E19" s="7" t="n"/>
@@ -6417,17 +6643,17 @@
     </row>
     <row r="20">
       <c r="A20" s="12" t="n">
-        <v>46487.625</v>
+        <v>46480.52083333334</v>
       </c>
       <c r="B20" s="7" t="n"/>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Renswoude 2</t>
+          <t>VRC 2</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Thuis</t>
+          <t>Uit</t>
         </is>
       </c>
       <c r="E20" s="7" t="n"/>
@@ -6436,17 +6662,17 @@
     </row>
     <row r="21">
       <c r="A21" s="12" t="n">
-        <v>46494.5</v>
+        <v>46487.625</v>
       </c>
       <c r="B21" s="7" t="n"/>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Candia '66 2</t>
+          <t>Renswoude 2</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Uit</t>
+          <t>Thuis</t>
         </is>
       </c>
       <c r="E21" s="7" t="n"/>
@@ -6455,17 +6681,17 @@
     </row>
     <row r="22">
       <c r="A22" s="12" t="n">
-        <v>46515.625</v>
+        <v>46494.5</v>
       </c>
       <c r="B22" s="7" t="n"/>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Roda '46 3</t>
+          <t>Candia '66 2</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Thuis</t>
+          <t>Uit</t>
         </is>
       </c>
       <c r="E22" s="7" t="n"/>
@@ -6474,17 +6700,17 @@
     </row>
     <row r="23">
       <c r="A23" s="12" t="n">
-        <v>46522.47916666666</v>
+        <v>46515.625</v>
       </c>
       <c r="B23" s="7" t="n"/>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>SVL 2</t>
+          <t>Roda '46 3</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Uit</t>
+          <t>Thuis</t>
         </is>
       </c>
       <c r="E23" s="7" t="n"/>
@@ -6493,17 +6719,17 @@
     </row>
     <row r="24">
       <c r="A24" s="12" t="n">
-        <v>46529.625</v>
+        <v>46522.47916666666</v>
       </c>
       <c r="B24" s="7" t="n"/>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Valleivogels 3</t>
+          <t>SVL 2</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Thuis</t>
+          <t>Uit</t>
         </is>
       </c>
       <c r="E24" s="7" t="n"/>
@@ -6511,13 +6737,23 @@
       <c r="G24" s="14" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="n"/>
+      <c r="A25" s="12" t="n">
+        <v>46529.625</v>
+      </c>
       <c r="B25" s="7" t="n"/>
-      <c r="C25" s="7" t="n"/>
-      <c r="D25" s="7" t="n"/>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Valleivogels 3</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Thuis</t>
+        </is>
+      </c>
       <c r="E25" s="7" t="n"/>
       <c r="F25" s="7" t="n"/>
-      <c r="G25" s="7" t="n"/>
+      <c r="G25" s="14" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="12" t="n"/>
@@ -6537,8 +6773,17 @@
       <c r="F27" s="7" t="n"/>
       <c r="G27" s="7" t="n"/>
     </row>
+    <row r="28">
+      <c r="A28" s="12" t="n"/>
+      <c r="B28" s="7" t="n"/>
+      <c r="C28" s="7" t="n"/>
+      <c r="D28" s="7" t="n"/>
+      <c r="E28" s="7" t="n"/>
+      <c r="F28" s="7" t="n"/>
+      <c r="G28" s="7" t="n"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:E200">
+  <conditionalFormatting sqref="D2:E201">
     <cfRule type="containsText" priority="1" operator="containsText" dxfId="2" text="(W)">
       <formula>NOT(ISERROR(SEARCH(("(W)"),(D2))))</formula>
     </cfRule>

</xml_diff>

<commit_message>
Stats bijgewerkt t/m 24-10-2026 (telefoon): 1-3 bij GVVV 2, Dennis en Kevin nieuw in selectie
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015WZFvXLYMKyAxjcVaLguDM
</commit_message>
<xml_diff>
--- a/data/WB3 Stats.xlsx
+++ b/data/WB3 Stats.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Selectie" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Training" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Competitie" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Oefen" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Wedstrijden" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selectie" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitie" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oefen" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wedstrijden" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Selectie'!$A$2:$N$37</definedName>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N48"/>
+  <dimension ref="A1:N49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.880000000000001" customWidth="1" style="15" min="2" max="2"/>
@@ -1671,15 +1671,28 @@
       <c r="N37" s="7" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="n"/>
-      <c r="B38" s="7" t="n"/>
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>Dennis</t>
+        </is>
+      </c>
+      <c r="B38" s="7">
+        <f>SUM(Competitie!B37:Q37)</f>
+        <v/>
+      </c>
       <c r="C38" s="7" t="n"/>
       <c r="D38" s="7" t="n"/>
       <c r="E38" s="7" t="n"/>
       <c r="F38" s="7" t="n"/>
       <c r="G38" s="7" t="n"/>
-      <c r="H38" s="7" t="n"/>
-      <c r="I38" s="7" t="n"/>
+      <c r="H38" s="7">
+        <f>SUM(Training!B37:P37)</f>
+        <v/>
+      </c>
+      <c r="I38" s="7">
+        <f>SUM(Oefen!B37:O37)</f>
+        <v/>
+      </c>
       <c r="J38" s="7" t="n"/>
       <c r="K38" s="7" t="n"/>
       <c r="L38" s="7" t="n"/>
@@ -1687,76 +1700,79 @@
       <c r="N38" s="7" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Kevin</t>
+        </is>
+      </c>
+      <c r="B39">
+        <f>SUM(Competitie!B38:Q38)</f>
+        <v/>
+      </c>
+      <c r="H39">
+        <f>SUM(Training!B38:P38)</f>
+        <v/>
+      </c>
+      <c r="I39">
+        <f>SUM(Oefen!B38:O38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>Totaal</t>
         </is>
       </c>
-      <c r="B39" s="8">
+      <c r="B40" s="8">
         <f>SUM(B3:B37)/990</f>
         <v/>
       </c>
-      <c r="C39" s="8">
+      <c r="C40" s="8">
         <f>SUM(C3:C37)</f>
         <v/>
       </c>
-      <c r="D39" s="8">
+      <c r="D40" s="8">
         <f>SUM(D3:D37)</f>
         <v/>
       </c>
-      <c r="E39" s="8">
+      <c r="E40" s="8">
         <f>SUM(E3:E37)</f>
         <v/>
       </c>
-      <c r="F39" s="8">
+      <c r="F40" s="8">
         <f>SUM(F3:F37)</f>
         <v/>
       </c>
-      <c r="G39" s="8">
+      <c r="G40" s="8">
         <f>SUM(G3:G37)</f>
         <v/>
       </c>
-      <c r="H39" s="8" t="n"/>
-      <c r="I39" s="8">
+      <c r="H40" s="8" t="n"/>
+      <c r="I40" s="8">
         <f>SUM(I3:I37)/990</f>
         <v/>
       </c>
-      <c r="J39" s="8">
+      <c r="J40" s="8">
         <f>SUM(J3:J37)</f>
         <v/>
       </c>
-      <c r="K39" s="8">
+      <c r="K40" s="8">
         <f>SUM(K3:K37)</f>
         <v/>
       </c>
-      <c r="L39" s="8">
+      <c r="L40" s="8">
         <f>SUM(L3:L37)</f>
         <v/>
       </c>
-      <c r="M39" s="8">
+      <c r="M40" s="8">
         <f>SUM(M3:M37)</f>
         <v/>
       </c>
-      <c r="N39" s="8">
+      <c r="N40" s="8">
         <f>SUM(N3:N37)</f>
         <v/>
       </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="7" t="n"/>
-      <c r="B40" s="7" t="n"/>
-      <c r="C40" s="7" t="n"/>
-      <c r="D40" s="7" t="n"/>
-      <c r="E40" s="7" t="n"/>
-      <c r="F40" s="7" t="n"/>
-      <c r="G40" s="7" t="n"/>
-      <c r="H40" s="7" t="n"/>
-      <c r="I40" s="7" t="n"/>
-      <c r="J40" s="7" t="n"/>
-      <c r="K40" s="7" t="n"/>
-      <c r="L40" s="7" t="n"/>
-      <c r="M40" s="7" t="n"/>
-      <c r="N40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="n"/>
@@ -1885,6 +1901,22 @@
       <c r="L48" s="7" t="n"/>
       <c r="M48" s="7" t="n"/>
       <c r="N48" s="7" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="n"/>
+      <c r="B49" s="7" t="n"/>
+      <c r="C49" s="7" t="n"/>
+      <c r="D49" s="7" t="n"/>
+      <c r="E49" s="7" t="n"/>
+      <c r="F49" s="7" t="n"/>
+      <c r="G49" s="7" t="n"/>
+      <c r="H49" s="7" t="n"/>
+      <c r="I49" s="7" t="n"/>
+      <c r="J49" s="7" t="n"/>
+      <c r="K49" s="7" t="n"/>
+      <c r="L49" s="7" t="n"/>
+      <c r="M49" s="7" t="n"/>
+      <c r="N49" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="$A$2:$N$37"/>
@@ -1902,7 +1934,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y50"/>
+  <dimension ref="A1:Y51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="8.880000000000001" customWidth="1" style="15" min="2" max="2"/>
@@ -3239,7 +3271,11 @@
       <c r="P36" s="7" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="n"/>
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>Dennis</t>
+        </is>
+      </c>
       <c r="B37" s="7" t="n"/>
       <c r="C37" s="7" t="n"/>
       <c r="D37" s="7" t="n"/>
@@ -3257,57 +3293,46 @@
       <c r="P37" s="7" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Kevin</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>Totaal</t>
         </is>
       </c>
-      <c r="B38" s="8">
+      <c r="B39" s="8">
         <f>SUM(B2:B36)</f>
         <v/>
       </c>
-      <c r="C38" s="8">
+      <c r="C39" s="8">
         <f>SUM(C2:C36)</f>
         <v/>
       </c>
-      <c r="D38" s="8">
+      <c r="D39" s="8">
         <f>SUM(D2:D36)</f>
         <v/>
       </c>
-      <c r="E38" s="8">
+      <c r="E39" s="8">
         <f>SUM(E2:E36)</f>
         <v/>
       </c>
-      <c r="F38" s="8">
+      <c r="F39" s="8">
         <f>SUM(F2:F36)</f>
         <v/>
       </c>
-      <c r="G38" s="8">
+      <c r="G39" s="8">
         <f>SUM(G2:G36)</f>
         <v/>
       </c>
-      <c r="H38" s="8">
+      <c r="H39" s="8">
         <f>SUM(H2:H36)</f>
         <v/>
       </c>
-      <c r="I38" s="7" t="n"/>
-      <c r="J38" s="7" t="n"/>
-      <c r="K38" s="7" t="n"/>
-      <c r="L38" s="7" t="n"/>
-      <c r="M38" s="7" t="n"/>
-      <c r="N38" s="7" t="n"/>
-      <c r="O38" s="7" t="n"/>
-      <c r="P38" s="7" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="7" t="n"/>
-      <c r="B39" s="7" t="n"/>
-      <c r="C39" s="7" t="n"/>
-      <c r="D39" s="7" t="n"/>
-      <c r="E39" s="7" t="n"/>
-      <c r="F39" s="7" t="n"/>
-      <c r="G39" s="8" t="n"/>
-      <c r="H39" s="7" t="n"/>
       <c r="I39" s="7" t="n"/>
       <c r="J39" s="7" t="n"/>
       <c r="K39" s="7" t="n"/>
@@ -3324,7 +3349,7 @@
       <c r="D40" s="7" t="n"/>
       <c r="E40" s="7" t="n"/>
       <c r="F40" s="7" t="n"/>
-      <c r="G40" s="7" t="n"/>
+      <c r="G40" s="8" t="n"/>
       <c r="H40" s="7" t="n"/>
       <c r="I40" s="7" t="n"/>
       <c r="J40" s="7" t="n"/>
@@ -3514,6 +3539,24 @@
       <c r="N50" s="7" t="n"/>
       <c r="O50" s="7" t="n"/>
       <c r="P50" s="7" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="n"/>
+      <c r="B51" s="7" t="n"/>
+      <c r="C51" s="7" t="n"/>
+      <c r="D51" s="7" t="n"/>
+      <c r="E51" s="7" t="n"/>
+      <c r="F51" s="7" t="n"/>
+      <c r="G51" s="7" t="n"/>
+      <c r="H51" s="7" t="n"/>
+      <c r="I51" s="7" t="n"/>
+      <c r="J51" s="7" t="n"/>
+      <c r="K51" s="7" t="n"/>
+      <c r="L51" s="7" t="n"/>
+      <c r="M51" s="7" t="n"/>
+      <c r="N51" s="7" t="n"/>
+      <c r="O51" s="7" t="n"/>
+      <c r="P51" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="$A$1:$P$36">
@@ -3539,7 +3582,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q47"/>
+  <dimension ref="A1:Q48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="6.25" customWidth="1" style="15" min="2" max="17"/>
@@ -4686,7 +4729,11 @@
       <c r="Q36" s="7" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="n"/>
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>Dennis</t>
+        </is>
+      </c>
       <c r="B37" s="7" t="n"/>
       <c r="C37" s="7" t="n"/>
       <c r="D37" s="7" t="n"/>
@@ -4705,47 +4752,35 @@
       <c r="Q37" s="7" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Kevin</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>Totaal</t>
         </is>
       </c>
-      <c r="B38" s="8">
+      <c r="B39" s="8">
         <f>SUM(B2:B36)</f>
         <v/>
       </c>
-      <c r="C38" s="8">
+      <c r="C39" s="8">
         <f>SUM(C2:C36)</f>
         <v/>
       </c>
-      <c r="D38" s="8">
+      <c r="D39" s="8">
         <f>SUM(D2:D36)</f>
         <v/>
       </c>
-      <c r="E38" s="8">
+      <c r="E39" s="8">
         <f>SUM(E2:E36)</f>
         <v/>
       </c>
-      <c r="F38" s="8" t="n"/>
-      <c r="G38" s="7" t="n"/>
-      <c r="H38" s="7" t="n"/>
-      <c r="I38" s="7" t="n"/>
-      <c r="J38" s="7" t="n"/>
-      <c r="K38" s="7" t="n"/>
-      <c r="L38" s="7" t="n"/>
-      <c r="M38" s="7" t="n"/>
-      <c r="N38" s="7" t="n"/>
-      <c r="O38" s="7" t="n"/>
-      <c r="P38" s="7" t="n"/>
-      <c r="Q38" s="7" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="7" t="n"/>
-      <c r="B39" s="7" t="n"/>
-      <c r="C39" s="7" t="n"/>
-      <c r="D39" s="7" t="n"/>
-      <c r="E39" s="7" t="n"/>
-      <c r="F39" s="7" t="n"/>
+      <c r="F39" s="8" t="n"/>
       <c r="G39" s="7" t="n"/>
       <c r="H39" s="7" t="n"/>
       <c r="I39" s="7" t="n"/>
@@ -4910,6 +4945,25 @@
       <c r="P47" s="7" t="n"/>
       <c r="Q47" s="7" t="n"/>
     </row>
+    <row r="48">
+      <c r="A48" s="7" t="n"/>
+      <c r="B48" s="7" t="n"/>
+      <c r="C48" s="7" t="n"/>
+      <c r="D48" s="7" t="n"/>
+      <c r="E48" s="7" t="n"/>
+      <c r="F48" s="7" t="n"/>
+      <c r="G48" s="7" t="n"/>
+      <c r="H48" s="7" t="n"/>
+      <c r="I48" s="7" t="n"/>
+      <c r="J48" s="7" t="n"/>
+      <c r="K48" s="7" t="n"/>
+      <c r="L48" s="7" t="n"/>
+      <c r="M48" s="7" t="n"/>
+      <c r="N48" s="7" t="n"/>
+      <c r="O48" s="7" t="n"/>
+      <c r="P48" s="7" t="n"/>
+      <c r="Q48" s="7" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4921,7 +4975,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q47"/>
+  <dimension ref="A1:Q48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="6.25" customWidth="1" style="15" min="2" max="17"/>
@@ -5900,7 +5954,11 @@
       <c r="Q36" s="7" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="n"/>
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>Dennis</t>
+        </is>
+      </c>
       <c r="B37" s="7" t="n"/>
       <c r="C37" s="7" t="n"/>
       <c r="D37" s="7" t="n"/>
@@ -5919,34 +5977,22 @@
       <c r="Q37" s="7" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="n"/>
-      <c r="B38" s="7">
-        <f>SUM(B2:B36)</f>
-        <v/>
-      </c>
-      <c r="C38" s="7">
-        <f>SUM(C2:C36)</f>
-        <v/>
-      </c>
-      <c r="D38" s="7" t="n"/>
-      <c r="E38" s="7" t="n"/>
-      <c r="F38" s="7" t="n"/>
-      <c r="G38" s="7" t="n"/>
-      <c r="H38" s="7" t="n"/>
-      <c r="I38" s="7" t="n"/>
-      <c r="J38" s="7" t="n"/>
-      <c r="K38" s="7" t="n"/>
-      <c r="L38" s="7" t="n"/>
-      <c r="M38" s="7" t="n"/>
-      <c r="N38" s="7" t="n"/>
-      <c r="O38" s="7" t="n"/>
-      <c r="P38" s="7" t="n"/>
-      <c r="Q38" s="7" t="n"/>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Kevin</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n"/>
-      <c r="B39" s="7" t="n"/>
-      <c r="C39" s="7" t="n"/>
+      <c r="B39" s="7">
+        <f>SUM(B2:B36)</f>
+        <v/>
+      </c>
+      <c r="C39" s="7">
+        <f>SUM(C2:C36)</f>
+        <v/>
+      </c>
       <c r="D39" s="7" t="n"/>
       <c r="E39" s="7" t="n"/>
       <c r="F39" s="7" t="n"/>
@@ -6113,6 +6159,25 @@
       <c r="O47" s="7" t="n"/>
       <c r="P47" s="7" t="n"/>
       <c r="Q47" s="7" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="n"/>
+      <c r="B48" s="7" t="n"/>
+      <c r="C48" s="7" t="n"/>
+      <c r="D48" s="7" t="n"/>
+      <c r="E48" s="7" t="n"/>
+      <c r="F48" s="7" t="n"/>
+      <c r="G48" s="7" t="n"/>
+      <c r="H48" s="7" t="n"/>
+      <c r="I48" s="7" t="n"/>
+      <c r="J48" s="7" t="n"/>
+      <c r="K48" s="7" t="n"/>
+      <c r="L48" s="7" t="n"/>
+      <c r="M48" s="7" t="n"/>
+      <c r="N48" s="7" t="n"/>
+      <c r="O48" s="7" t="n"/>
+      <c r="P48" s="7" t="n"/>
+      <c r="Q48" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Training 29 oktober toegevoegd (telefoon)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015WZFvXLYMKyAxjcVaLguDM
</commit_message>
<xml_diff>
--- a/data/WB3 Stats.xlsx
+++ b/data/WB3 Stats.xlsx
@@ -1700,20 +1700,20 @@
       <c r="N38" s="7" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="0" t="inlineStr">
         <is>
           <t>Kevin</t>
         </is>
       </c>
-      <c r="B39">
+      <c r="B39" s="0">
         <f>SUM(Competitie!B38:Q38)</f>
         <v/>
       </c>
-      <c r="H39">
+      <c r="H39" s="0">
         <f>SUM(Training!B38:P38)</f>
         <v/>
       </c>
-      <c r="I39">
+      <c r="I39" s="0">
         <f>SUM(Oefen!B38:O38)</f>
         <v/>
       </c>
@@ -2038,7 +2038,9 @@
         <v>0</v>
       </c>
       <c r="I2" s="7" t="n"/>
-      <c r="J2" s="7" t="n"/>
+      <c r="J2" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K2" s="7" t="n"/>
       <c r="L2" s="7" t="n"/>
       <c r="M2" s="7" t="n"/>
@@ -2074,7 +2076,9 @@
         <v>0</v>
       </c>
       <c r="I3" s="7" t="n"/>
-      <c r="J3" s="7" t="n"/>
+      <c r="J3" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K3" s="7" t="n"/>
       <c r="L3" s="7" t="n"/>
       <c r="M3" s="7" t="n"/>
@@ -2110,7 +2114,9 @@
         <v>0</v>
       </c>
       <c r="I4" s="7" t="n"/>
-      <c r="J4" s="7" t="n"/>
+      <c r="J4" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K4" s="7" t="n"/>
       <c r="L4" s="7" t="n"/>
       <c r="M4" s="7" t="n"/>
@@ -2146,7 +2152,9 @@
         <v>0</v>
       </c>
       <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
+      <c r="J5" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K5" s="7" t="n"/>
       <c r="L5" s="7" t="n"/>
       <c r="M5" s="7" t="n"/>
@@ -2182,7 +2190,9 @@
         <v>1</v>
       </c>
       <c r="I6" s="7" t="n"/>
-      <c r="J6" s="7" t="n"/>
+      <c r="J6" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K6" s="7" t="n"/>
       <c r="L6" s="7" t="n"/>
       <c r="M6" s="7" t="n"/>
@@ -2218,7 +2228,9 @@
         <v>1</v>
       </c>
       <c r="I7" s="7" t="n"/>
-      <c r="J7" s="7" t="n"/>
+      <c r="J7" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="K7" s="7" t="n"/>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7" t="n"/>
@@ -2254,7 +2266,9 @@
         <v>0</v>
       </c>
       <c r="I8" s="7" t="n"/>
-      <c r="J8" s="7" t="n"/>
+      <c r="J8" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K8" s="7" t="n"/>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7" t="n"/>
@@ -2290,7 +2304,9 @@
         <v>1</v>
       </c>
       <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
+      <c r="J9" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="K9" s="7" t="n"/>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7" t="n"/>
@@ -2326,7 +2342,9 @@
         <v>0</v>
       </c>
       <c r="I10" s="7" t="n"/>
-      <c r="J10" s="7" t="n"/>
+      <c r="J10" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="K10" s="7" t="n"/>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7" t="n"/>
@@ -2362,7 +2380,9 @@
         <v>0</v>
       </c>
       <c r="I11" s="7" t="n"/>
-      <c r="J11" s="7" t="n"/>
+      <c r="J11" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K11" s="7" t="n"/>
       <c r="L11" s="7" t="n"/>
       <c r="M11" s="7" t="n"/>
@@ -2398,7 +2418,9 @@
         <v>0</v>
       </c>
       <c r="I12" s="7" t="n"/>
-      <c r="J12" s="7" t="n"/>
+      <c r="J12" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K12" s="7" t="n"/>
       <c r="L12" s="7" t="n"/>
       <c r="M12" s="7" t="n"/>
@@ -2434,7 +2456,9 @@
         <v>0</v>
       </c>
       <c r="I13" s="7" t="n"/>
-      <c r="J13" s="7" t="n"/>
+      <c r="J13" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K13" s="7" t="n"/>
       <c r="L13" s="7" t="n"/>
       <c r="M13" s="7" t="n"/>
@@ -2470,7 +2494,9 @@
         <v>0</v>
       </c>
       <c r="I14" s="7" t="n"/>
-      <c r="J14" s="7" t="n"/>
+      <c r="J14" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K14" s="7" t="n"/>
       <c r="L14" s="7" t="n"/>
       <c r="M14" s="7" t="n"/>
@@ -2506,7 +2532,9 @@
         <v>0</v>
       </c>
       <c r="I15" s="7" t="n"/>
-      <c r="J15" s="7" t="n"/>
+      <c r="J15" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K15" s="7" t="n"/>
       <c r="L15" s="7" t="n"/>
       <c r="M15" s="7" t="n"/>
@@ -2542,7 +2570,9 @@
         <v>1</v>
       </c>
       <c r="I16" s="7" t="n"/>
-      <c r="J16" s="7" t="n"/>
+      <c r="J16" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K16" s="7" t="n"/>
       <c r="L16" s="7" t="n"/>
       <c r="M16" s="7" t="n"/>
@@ -2578,7 +2608,9 @@
         <v>1</v>
       </c>
       <c r="I17" s="7" t="n"/>
-      <c r="J17" s="7" t="n"/>
+      <c r="J17" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="K17" s="7" t="n"/>
       <c r="L17" s="7" t="n"/>
       <c r="M17" s="7" t="n"/>
@@ -2614,7 +2646,9 @@
         <v>1</v>
       </c>
       <c r="I18" s="7" t="n"/>
-      <c r="J18" s="7" t="n"/>
+      <c r="J18" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K18" s="7" t="n"/>
       <c r="L18" s="7" t="n"/>
       <c r="M18" s="7" t="n"/>
@@ -2650,7 +2684,9 @@
         <v>1</v>
       </c>
       <c r="I19" s="7" t="n"/>
-      <c r="J19" s="7" t="n"/>
+      <c r="J19" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="K19" s="7" t="n"/>
       <c r="L19" s="7" t="n"/>
       <c r="M19" s="7" t="n"/>
@@ -2686,7 +2722,9 @@
         <v>0</v>
       </c>
       <c r="I20" s="7" t="n"/>
-      <c r="J20" s="7" t="n"/>
+      <c r="J20" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="K20" s="7" t="n"/>
       <c r="L20" s="7" t="n"/>
       <c r="M20" s="7" t="n"/>
@@ -2722,7 +2760,9 @@
         <v>1</v>
       </c>
       <c r="I21" s="7" t="n"/>
-      <c r="J21" s="7" t="n"/>
+      <c r="J21" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="K21" s="7" t="n"/>
       <c r="L21" s="7" t="n"/>
       <c r="M21" s="7" t="n"/>
@@ -2758,7 +2798,9 @@
         <v>0</v>
       </c>
       <c r="I22" s="7" t="n"/>
-      <c r="J22" s="7" t="n"/>
+      <c r="J22" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K22" s="7" t="n"/>
       <c r="L22" s="7" t="n"/>
       <c r="M22" s="7" t="n"/>
@@ -2794,7 +2836,9 @@
         <v>0</v>
       </c>
       <c r="I23" s="7" t="n"/>
-      <c r="J23" s="7" t="n"/>
+      <c r="J23" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K23" s="7" t="n"/>
       <c r="L23" s="7" t="n"/>
       <c r="M23" s="7" t="n"/>
@@ -2830,7 +2874,9 @@
         <v>0</v>
       </c>
       <c r="I24" s="7" t="n"/>
-      <c r="J24" s="7" t="n"/>
+      <c r="J24" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K24" s="7" t="n"/>
       <c r="L24" s="7" t="n"/>
       <c r="M24" s="7" t="n"/>
@@ -2866,7 +2912,9 @@
         <v>0</v>
       </c>
       <c r="I25" s="7" t="n"/>
-      <c r="J25" s="7" t="n"/>
+      <c r="J25" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K25" s="7" t="n"/>
       <c r="L25" s="7" t="n"/>
       <c r="M25" s="7" t="n"/>
@@ -2902,7 +2950,9 @@
         <v>1</v>
       </c>
       <c r="I26" s="7" t="n"/>
-      <c r="J26" s="7" t="n"/>
+      <c r="J26" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K26" s="7" t="n"/>
       <c r="L26" s="7" t="n"/>
       <c r="M26" s="7" t="n"/>
@@ -2938,7 +2988,9 @@
         <v>0</v>
       </c>
       <c r="I27" s="7" t="n"/>
-      <c r="J27" s="7" t="n"/>
+      <c r="J27" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K27" s="7" t="n"/>
       <c r="L27" s="7" t="n"/>
       <c r="M27" s="7" t="n"/>
@@ -2974,7 +3026,9 @@
         <v>1</v>
       </c>
       <c r="I28" s="7" t="n"/>
-      <c r="J28" s="7" t="n"/>
+      <c r="J28" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K28" s="7" t="n"/>
       <c r="L28" s="7" t="n"/>
       <c r="M28" s="7" t="n"/>
@@ -3010,7 +3064,9 @@
         <v>0</v>
       </c>
       <c r="I29" s="7" t="n"/>
-      <c r="J29" s="7" t="n"/>
+      <c r="J29" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K29" s="7" t="n"/>
       <c r="L29" s="7" t="n"/>
       <c r="M29" s="7" t="n"/>
@@ -3046,7 +3102,9 @@
         <v>0</v>
       </c>
       <c r="I30" s="7" t="n"/>
-      <c r="J30" s="7" t="n"/>
+      <c r="J30" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K30" s="7" t="n"/>
       <c r="L30" s="7" t="n"/>
       <c r="M30" s="7" t="n"/>
@@ -3082,7 +3140,9 @@
         <v>0</v>
       </c>
       <c r="I31" s="7" t="n"/>
-      <c r="J31" s="7" t="n"/>
+      <c r="J31" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K31" s="7" t="n"/>
       <c r="L31" s="7" t="n"/>
       <c r="M31" s="7" t="n"/>
@@ -3118,7 +3178,9 @@
         <v>0</v>
       </c>
       <c r="I32" s="7" t="n"/>
-      <c r="J32" s="7" t="n"/>
+      <c r="J32" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K32" s="7" t="n"/>
       <c r="L32" s="7" t="n"/>
       <c r="M32" s="7" t="n"/>
@@ -3154,7 +3216,9 @@
         <v>0</v>
       </c>
       <c r="I33" s="7" t="n"/>
-      <c r="J33" s="7" t="n"/>
+      <c r="J33" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="K33" s="7" t="n"/>
       <c r="L33" s="7" t="n"/>
       <c r="M33" s="7" t="n"/>
@@ -3190,7 +3254,9 @@
         <v>0</v>
       </c>
       <c r="I34" s="7" t="n"/>
-      <c r="J34" s="7" t="n"/>
+      <c r="J34" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="K34" s="7" t="n"/>
       <c r="L34" s="7" t="n"/>
       <c r="M34" s="7" t="n"/>
@@ -3226,7 +3292,9 @@
         <v>0</v>
       </c>
       <c r="I35" s="7" t="n"/>
-      <c r="J35" s="7" t="n"/>
+      <c r="J35" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K35" s="7" t="n"/>
       <c r="L35" s="7" t="n"/>
       <c r="M35" s="7" t="n"/>
@@ -3262,7 +3330,9 @@
         <v>1</v>
       </c>
       <c r="I36" s="7" t="n"/>
-      <c r="J36" s="7" t="n"/>
+      <c r="J36" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="K36" s="7" t="n"/>
       <c r="L36" s="7" t="n"/>
       <c r="M36" s="7" t="n"/>
@@ -3284,7 +3354,9 @@
       <c r="G37" s="7" t="n"/>
       <c r="H37" s="7" t="n"/>
       <c r="I37" s="7" t="n"/>
-      <c r="J37" s="7" t="n"/>
+      <c r="J37" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="K37" s="7" t="n"/>
       <c r="L37" s="7" t="n"/>
       <c r="M37" s="7" t="n"/>
@@ -3293,10 +3365,13 @@
       <c r="P37" s="7" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="0" t="inlineStr">
         <is>
           <t>Kevin</t>
         </is>
+      </c>
+      <c r="J38" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -4752,7 +4827,7 @@
       <c r="Q37" s="7" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="0" t="inlineStr">
         <is>
           <t>Kevin</t>
         </is>
@@ -5977,7 +6052,7 @@
       <c r="Q37" s="7" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="0" t="inlineStr">
         <is>
           <t>Kevin</t>
         </is>

</xml_diff>